<commit_message>
Correct Monday night: ESPN roster flag is post-game only, Barkley active via operator status, corrected freeze and card, DECISIONS #55
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DRV9GgxaEbuX9GLrrgpBnz
</commit_message>
<xml_diff>
--- a/docs/weekly/SLATE_MNF_2026_W07.xlsx
+++ b/docs/weekly/SLATE_MNF_2026_W07.xlsx
@@ -486,7 +486,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Inputs used (UTC). ESPN game-summary Outs (5 names per team cap, not the official inactives): 2026-10-26T22:55:05Z. Sleeper status overlay (newer Out replaces the NFL row): 2026-10-26T22:54:57+00:00. nflverse depth charts: 2026-10-26T14:07:44Z; nflverse injuries: no timestamp in the feed. Lines: ESPN/DraftKings fetched 2026-10-26T22:55Z (no prices; the per-line last_updated_utc stamps run ahead of the fetch time and their zone is unverified, so no recency claim is made from them). Inactives: nflverse roster INA where the league's list has reached it, ESPN event-roster didNotPlay flags within 100 minutes of kickoff (they matched the official list 13 of 13 on a finished game), and the ESPN game-summary Outs (5 names per team); a team with no INA rows yet is pending, not healthy. A Sleeper status that disagrees with the ESPN flag is listed in the injury audit. Code: git 9dd1647.</t>
+          <t>Inputs used (UTC). ESPN game-summary Outs (5 names per team cap, not the official inactives): 2026-10-26T23:07:53Z. Sleeper status overlay (newer Out replaces the NFL row): 2026-10-26T23:07:45+00:00. nflverse depth charts: 2026-10-26T14:07:44Z; nflverse injuries: no timestamp in the feed. Lines: ESPN/DraftKings fetched 2026-10-26T23:08Z (no prices; the per-line last_updated_utc stamps run ahead of the fetch time and their zone is unverified, so no recency claim is made from them). Inactives: nflverse roster INA where the league's list has reached it, and the ESPN game-summary Outs (5 names per team). The ESPN event-roster didNotPlay flag is a post-game record only: before kickoff it is not the inactive list (it listed Barkley inactive when the league listed him active); a team with no INA rows yet is pending, not healthy. A Sleeper status that disagrees with the ESPN flag is listed in the injury audit. Code: git 4e68902.</t>
         </is>
       </c>
     </row>
@@ -512,8 +512,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
   </cols>
@@ -661,39 +661,39 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DAL@PHI: Jake Ferguson anytime TD + DAL@PHI: Dak Prescott pass TD 1+</t>
+          <t>DAL@PHI: Saquon Barkley anytime TD + DAL@PHI: Dak Prescott pass TD 1+</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.147</v>
+        <v>0.149</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>0.178</v>
+        <v>0.18</v>
       </c>
       <c r="D13" t="n">
-        <v>581</v>
+        <v>572</v>
       </c>
       <c r="E13" t="n">
-        <v>662</v>
+        <v>653</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DAL@PHI: Makai Lemon anytime TD + DAL@PHI: Dak Prescott pass TD 1+</t>
+          <t>DAL@PHI: Jake Ferguson anytime TD + DAL@PHI: Dak Prescott pass TD 1+</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.138</v>
+        <v>0.147</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>0.167</v>
+        <v>0.178</v>
       </c>
       <c r="D14" t="n">
-        <v>626</v>
+        <v>580</v>
       </c>
       <c r="E14" t="n">
-        <v>714</v>
+        <v>662</v>
       </c>
     </row>
     <row r="15"/>
@@ -797,67 +797,67 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="D23" t="n">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="E23" t="n">
-        <v>1323</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Jake Ferguson anytime TD</t>
+          <t>DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Saquon Barkley anytime TD + DAL@PHI: Dak Prescott pass TD 1+</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.063</v>
+        <v>0.068</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>0.057</v>
+        <v>0.08199999999999999</v>
       </c>
       <c r="D24" t="n">
-        <v>1475</v>
+        <v>1375</v>
       </c>
       <c r="E24" t="n">
-        <v>1664</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Makai Lemon anytime TD + DAL@PHI: Dak Prescott pass TD 1+</t>
+          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Jake Ferguson anytime TD</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.062</v>
+        <v>0.064</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>0.075</v>
+        <v>0.057</v>
       </c>
       <c r="D25" t="n">
-        <v>1517</v>
+        <v>1474</v>
       </c>
       <c r="E25" t="n">
-        <v>1711</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: Ryan Flournoy anytime TD + DAL@PHI: Jake Ferguson anytime TD</t>
+          <t>DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Makai Lemon anytime TD + DAL@PHI: Dak Prescott pass TD 1+</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.042</v>
+        <v>0.058</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="D26" t="n">
-        <v>2304</v>
+        <v>1620</v>
       </c>
       <c r="E26" t="n">
-        <v>2593</v>
+        <v>1827</v>
       </c>
     </row>
     <row r="27"/>
@@ -951,77 +951,77 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Ryan Flournoy anytime TD + DAL@PHI: Makai Lemon anytime TD</t>
+          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Saquon Barkley anytime TD + DAL@PHI: Ryan Flournoy anytime TD</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="C35" s="6" t="n">
         <v>0.017</v>
       </c>
-      <c r="C35" s="6" t="n">
-        <v>0.016</v>
-      </c>
       <c r="D35" t="n">
-        <v>5678</v>
+        <v>5263</v>
       </c>
       <c r="E35" t="n">
-        <v>6372</v>
+        <v>5907</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Makai Lemon anytime TD + DAL@PHI: Jake Ferguson anytime TD</t>
+          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Ryan Flournoy anytime TD + DAL@PHI: Makai Lemon anytime TD</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="C36" s="6" t="n">
         <v>0.014</v>
       </c>
-      <c r="C36" s="6" t="n">
-        <v>0.013</v>
-      </c>
       <c r="D36" t="n">
-        <v>6980</v>
+        <v>6163</v>
       </c>
       <c r="E36" t="n">
-        <v>7830</v>
+        <v>6915</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Ryan Flournoy anytime TD + DAL@PHI: Jake Ferguson anytime TD</t>
+          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Saquon Barkley anytime TD + DAL@PHI: Jake Ferguson anytime TD</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C37" s="6" t="n">
         <v>0.014</v>
       </c>
-      <c r="C37" s="6" t="n">
-        <v>0.013</v>
-      </c>
       <c r="D37" t="n">
-        <v>7037</v>
+        <v>6510</v>
       </c>
       <c r="E37" t="n">
-        <v>7893</v>
+        <v>7303</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: Ryan Flournoy anytime TD + DAL@PHI: Makai Lemon anytime TD + DAL@PHI: Jake Ferguson anytime TD</t>
+          <t>DAL@PHI: Dak Prescott pass TD 2+ + DAL@PHI: CeeDee Lamb anytime TD + DAL@PHI: Ryan Flournoy anytime TD + DAL@PHI: Jake Ferguson anytime TD</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.014</v>
       </c>
       <c r="C38" s="6" t="n">
-        <v>0.008</v>
+        <v>0.013</v>
       </c>
       <c r="D38" t="n">
-        <v>11166</v>
+        <v>7008</v>
       </c>
       <c r="E38" t="n">
-        <v>12518</v>
+        <v>7861</v>
       </c>
     </row>
     <row r="39"/>
@@ -1269,13 +1269,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="57" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1289,7 +1289,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>3 players have posted lines but no projection row (not on the 2026 stats universe, injured/exempt, or name mismatch). Nothing is published for them:</t>
+          <t>1 players have posted lines but no projection row (not on the 2026 stats universe, injured/exempt, or name mismatch). Nothing is published for them:</t>
         </is>
       </c>
     </row>
@@ -1337,79 +1337,69 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Marquise Brown</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DAL@PHI</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>reception_yds, receptions</t>
-        </is>
-      </c>
-    </row>
+    <row r="6"/>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Saquon Barkley</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DAL@PHI</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>reception_yds, receptions, rush_attempts, rush_yds</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Withheld on purpose (no line, touchdown or parlay leg):</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Withheld on purpose (no line, touchdown or parlay leg):</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Josh Jacobs</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>RB1 on the depth chart and ACT on the roster with no 2026 games and no projection row (book lines posted; role unknown)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>player</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>team</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>reason</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MarShawn Lloyd</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GB backfield shares are unpriced while Jacobs is missing</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Josh Jacobs</t>
+          <t>Kaleb Johnson</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1419,14 +1409,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RB1 on the depth chart and ACT on the roster with no 2026 games and no projection row (book lines posted; role unknown)</t>
+          <t>GB backfield shares are unpriced while Jacobs is missing</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MarShawn Lloyd</t>
+          <t>Pierre Strong</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1443,7 +1433,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kaleb Johnson</t>
+          <t>Chris Brooks</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1452,40 +1442,6 @@
         </is>
       </c>
       <c r="C13" t="inlineStr">
-        <is>
-          <t>GB backfield shares are unpriced while Jacobs is missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Pierre Strong</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>GB backfield shares are unpriced while Jacobs is missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Chris Brooks</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
         <is>
           <t>GB backfield shares are unpriced while Jacobs is missing</t>
         </is>
@@ -1691,20 +1647,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DAL 24.0, PHI 19.5</t>
+          <t>DAL 24.0, PHI 19.6</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>DAL 62% / PHI 38%</t>
+          <t>DAL 63% / PHI 37%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>43.5</v>
+        <v>43.6</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>DAL 23.2, PHI 23.9</t>
+          <t>DAL 23.2, PHI 23.8</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1806,7 +1762,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Already played: KC@SEA final KC 3, SEA 20 (market SEA -3.0, total 43.5; projected 20.1-23.3).</t>
+          <t>Already played: KC@SEA final KC 3, SEA 20 (market SEA -3.0, total 43.5; projected 20.2-23.3).</t>
         </is>
       </c>
     </row>
@@ -7220,7 +7176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -7346,13 +7302,13 @@
         <v>23.8</v>
       </c>
       <c r="F6" t="n">
-        <v>260.6</v>
+        <v>259.3</v>
       </c>
       <c r="G6" t="n">
         <v>1.37</v>
       </c>
       <c r="H6" t="n">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="I6" t="n">
         <v>0.16</v>
@@ -7387,28 +7343,28 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>20.5</v>
+        <v>20.6</v>
       </c>
       <c r="F7" t="n">
-        <v>216</v>
+        <v>207.9</v>
       </c>
       <c r="G7" t="n">
         <v>1.35</v>
       </c>
       <c r="H7" t="n">
-        <v>15.1</v>
+        <v>7.7</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>0.09</v>
+        <v>0.05</v>
       </c>
       <c r="K7" t="n">
-        <v>8.699999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="L7" t="n">
-        <v>14.7</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="8"/>
@@ -7514,7 +7470,7 @@
         <v>15.9</v>
       </c>
       <c r="F11" t="n">
-        <v>64.09999999999999</v>
+        <v>63.8</v>
       </c>
       <c r="G11" t="n">
         <v>0.87</v>
@@ -7523,7 +7479,7 @@
         <v>2.8</v>
       </c>
       <c r="I11" t="n">
-        <v>17.7</v>
+        <v>17.8</v>
       </c>
       <c r="J11" t="n">
         <v>0.11</v>
@@ -7561,90 +7517,90 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>15.7</v>
+        <v>11.3</v>
       </c>
       <c r="F12" t="n">
-        <v>65.2</v>
+        <v>43.9</v>
       </c>
       <c r="G12" t="n">
-        <v>0.36</v>
+        <v>0.28</v>
       </c>
       <c r="H12" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="I12" t="n">
-        <v>27.2</v>
+        <v>22.5</v>
       </c>
       <c r="J12" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="L12" t="n">
-        <v>3.1</v>
+        <v>2.5</v>
       </c>
       <c r="M12" t="n">
-        <v>16</v>
+        <v>12.2</v>
       </c>
       <c r="N12" t="n">
-        <v>15.8</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tyler Goodson</t>
+          <t>Saquon Barkley</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>DAL</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>PHI</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>3.2</v>
+        <v>6.8</v>
       </c>
       <c r="F13" t="n">
-        <v>13.2</v>
+        <v>34</v>
       </c>
       <c r="G13" t="n">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6</v>
+        <v>2.1</v>
       </c>
       <c r="I13" t="n">
-        <v>4.8</v>
+        <v>15.6</v>
       </c>
       <c r="J13" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>0.13</v>
+        <v>0.23</v>
       </c>
       <c r="L13" t="n">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="M13" t="n">
-        <v>3.3</v>
+        <v>8.6</v>
       </c>
       <c r="N13" t="n">
-        <v>3.2</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hunter Luepke</t>
+          <t>Tyler Goodson</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7661,152 +7617,158 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M14" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="N14" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Hunter Luepke</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
         <v>1.1</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F15" t="n">
         <v>4.9</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G15" t="n">
         <v>0.04</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H15" t="n">
         <v>0.5</v>
       </c>
-      <c r="I14" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="J14" t="n">
+      <c r="I15" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="J15" t="n">
         <v>0.02</v>
       </c>
-      <c r="K14" s="6" t="n">
+      <c r="K15" s="6" t="n">
         <v>0.06</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L15" t="n">
         <v>0.4</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M15" t="n">
         <v>1.8</v>
       </c>
-      <c r="N14" t="inlineStr"/>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="N15" t="inlineStr"/>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Wide receivers</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>player</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>team</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>opp</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>p_active</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>tgt_mean</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>rec_mean</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>rec_yds_mean</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>rec_td_mean</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>any_td_pct</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>league_ev</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>ppr</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>dk</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>CeeDee Lamb</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="F18" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="G18" t="n">
-        <v>84.59999999999999</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="I18" s="6" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="J18" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="K18" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="L18" t="n">
-        <v>17.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>George Pickens</t>
+          <t>CeeDee Lamb</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7820,148 +7782,148 @@
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>9</v>
+        <v>10.9</v>
       </c>
       <c r="F19" t="n">
-        <v>5.5</v>
+        <v>6.7</v>
       </c>
       <c r="G19" t="n">
-        <v>73.40000000000001</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>0.31</v>
+        <v>0.42</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.27</v>
+        <v>0.36</v>
       </c>
       <c r="J19" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="K19" t="n">
-        <v>14.7</v>
+        <v>17.8</v>
       </c>
       <c r="L19" t="n">
-        <v>13.9</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Darius Cooper</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
       <c r="D20" s="6" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F20" t="n">
-        <v>1.8</v>
+        <v>5.5</v>
       </c>
       <c r="G20" t="n">
-        <v>24.7</v>
+        <v>73.3</v>
       </c>
       <c r="H20" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.25</v>
+        <v>0.27</v>
       </c>
       <c r="J20" t="n">
         <v>1.7</v>
       </c>
       <c r="K20" t="n">
-        <v>5.9</v>
+        <v>14.7</v>
       </c>
       <c r="L20" t="n">
-        <v>5.9</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ryan Flournoy</t>
+          <t>Darius Cooper</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>DAL</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>PHI</t>
         </is>
       </c>
       <c r="D21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>5.8</v>
+        <v>2.6</v>
       </c>
       <c r="F21" t="n">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="G21" t="n">
-        <v>39.8</v>
+        <v>20.5</v>
       </c>
       <c r="H21" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="J21" t="n">
         <v>1.5</v>
       </c>
       <c r="K21" t="n">
-        <v>9</v>
+        <v>5.1</v>
       </c>
       <c r="L21" t="n">
-        <v>9</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Makai Lemon</t>
+          <t>Ryan Flournoy</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>PHI</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>DAL</t>
         </is>
       </c>
       <c r="D22" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>7.8</v>
+        <v>5.8</v>
       </c>
       <c r="F22" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="G22" t="n">
-        <v>49.7</v>
+        <v>39.8</v>
       </c>
       <c r="H22" t="n">
         <v>0.24</v>
@@ -7973,16 +7935,16 @@
         <v>1.4</v>
       </c>
       <c r="K22" t="n">
-        <v>11</v>
+        <v>8.9</v>
       </c>
       <c r="L22" t="n">
-        <v>11</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Elijah Moore</t>
+          <t>Makai Lemon</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7999,402 +7961,406 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>1.6</v>
+        <v>6.6</v>
       </c>
       <c r="F23" t="n">
-        <v>0.9</v>
+        <v>3.9</v>
       </c>
       <c r="G23" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="H23" t="n">
-        <v>0.05</v>
+        <v>0.21</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>0.06</v>
+        <v>0.2</v>
       </c>
       <c r="J23" t="n">
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
       <c r="K23" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="L23" t="inlineStr"/>
+        <v>9.300000000000001</v>
+      </c>
+      <c r="L23" t="n">
+        <v>9.300000000000001</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Jonathan Mingo</t>
+          <t>Marquise Brown</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
       <c r="D24" s="6" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="E24" t="n">
-        <v>1.2</v>
+        <v>2.7</v>
       </c>
       <c r="F24" t="n">
-        <v>0.7</v>
+        <v>1.6</v>
       </c>
       <c r="G24" t="n">
-        <v>9.1</v>
+        <v>19.8</v>
       </c>
       <c r="H24" t="n">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="J24" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="K24" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
+        <v>4.3</v>
+      </c>
+      <c r="L24" t="n">
+        <v>4.1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>Jonathan Mingo</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G25" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K25" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Elijah Moore</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G26" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Britain Covey</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="D25" s="6" t="n">
+      <c r="D27" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="E25" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G25" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I25" s="6" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="J25" t="n">
+      <c r="E27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J27" t="n">
         <v>0.1</v>
       </c>
-      <c r="K25" t="n">
-        <v>1</v>
-      </c>
-      <c r="L25" t="inlineStr"/>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="K27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Tight ends</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>player</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>team</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>opp</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>p_active</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>tgt_mean</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>rec_mean</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>rec_yds_mean</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>rec_td_mean</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>any_td_pct</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>league_ev</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="K30" s="4" t="inlineStr">
         <is>
           <t>ppr</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="L30" s="4" t="inlineStr">
         <is>
           <t>dk</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Dallas Goedert</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E29" t="n">
-        <v>9.300000000000001</v>
-      </c>
-      <c r="F29" t="n">
-        <v>6</v>
-      </c>
-      <c r="G29" t="n">
-        <v>63.1</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="I29" s="6" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="J29" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="K29" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="L29" t="n">
-        <v>13.8</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Zach Ertz</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="F30" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="G30" t="n">
-        <v>43.1</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="I30" s="6" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="J30" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="K30" t="n">
-        <v>10</v>
-      </c>
-      <c r="L30" t="n">
-        <v>9.9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jake Ferguson</t>
+          <t>Dallas Goedert</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
       <c r="D31" s="6" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="E31" t="n">
-        <v>5.5</v>
+        <v>7.9</v>
       </c>
       <c r="F31" t="n">
-        <v>3.7</v>
+        <v>5.1</v>
       </c>
       <c r="G31" t="n">
-        <v>33.7</v>
+        <v>52.1</v>
       </c>
       <c r="H31" t="n">
-        <v>0.2</v>
+        <v>0.34</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>0.18</v>
+        <v>0.29</v>
       </c>
       <c r="J31" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="K31" t="n">
-        <v>8.300000000000001</v>
+        <v>12.4</v>
       </c>
       <c r="L31" t="n">
-        <v>8.199999999999999</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Brevyn Spann-Ford</t>
+          <t>Zach Ertz</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
           <t>DAL</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>PHI</t>
         </is>
       </c>
       <c r="D32" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1.7</v>
+        <v>5.6</v>
       </c>
       <c r="F32" t="n">
-        <v>1.1</v>
+        <v>3.5</v>
       </c>
       <c r="G32" t="n">
-        <v>11</v>
+        <v>35.4</v>
       </c>
       <c r="H32" t="n">
-        <v>0.06</v>
+        <v>0.22</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>0.06</v>
+        <v>0.2</v>
       </c>
       <c r="J32" t="n">
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
       <c r="K32" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L32" t="inlineStr"/>
+        <v>8.4</v>
+      </c>
+      <c r="L32" t="n">
+        <v>8.300000000000001</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Johnny Mundt</t>
+          <t>Jake Ferguson</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
           <t>PHI</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>DAL</t>
         </is>
       </c>
       <c r="D33" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1.6</v>
+        <v>5.5</v>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>3.7</v>
       </c>
       <c r="G33" t="n">
-        <v>10.4</v>
+        <v>33.5</v>
       </c>
       <c r="H33" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>0.06</v>
+        <v>0.18</v>
       </c>
       <c r="J33" t="n">
-        <v>0.3</v>
+        <v>1.2</v>
       </c>
       <c r="K33" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="L33" t="inlineStr"/>
+        <v>8.300000000000001</v>
+      </c>
+      <c r="L33" t="n">
+        <v>8.199999999999999</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Luke Schoonmaker</t>
+          <t>Brevyn Spann-Ford</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -8411,31 +8377,115 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="F34" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="G34" t="n">
-        <v>5.7</v>
+        <v>10.9</v>
       </c>
       <c r="H34" t="n">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="I34" s="6" t="n">
         <v>0.06</v>
       </c>
       <c r="J34" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K34" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Johnny Mundt</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G35" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K35" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Luke Schoonmaker</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G36" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J36" t="n">
         <v>0.1</v>
       </c>
-      <c r="K34" t="n">
+      <c r="K36" t="n">
         <v>1.3</v>
       </c>
-      <c r="L34" t="inlineStr"/>
-    </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="L36" t="inlineStr"/>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Kickers (this league: FG 3, XP 1; ranked by team implied points, the only validated signal; differences are within noise): DAL 7.5; PHI 6.9</t>
         </is>
@@ -8452,7 +8502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -8556,16 +8606,16 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.637</v>
+        <v>0.643</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.637</v>
+        <v>0.643</v>
       </c>
       <c r="G5" t="n">
-        <v>-176</v>
+        <v>-180</v>
       </c>
       <c r="H5" t="n">
-        <v>-132</v>
+        <v>-135</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>1</v>
@@ -8579,84 +8629,84 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dameon Pierce</t>
+          <t>CeeDee Lamb</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.418</v>
+        <v>0.357</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.418</v>
+        <v>0.357</v>
       </c>
       <c r="G6" t="n">
-        <v>139</v>
+        <v>180</v>
       </c>
       <c r="H6" t="n">
-        <v>168</v>
+        <v>214</v>
       </c>
       <c r="I6" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>fill-in QB (Tanner McKee) red-team downgrade</t>
+          <t>opp QB: fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CeeDee Lamb</t>
+          <t>Dameon Pierce</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.356</v>
+        <v>0.348</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.356</v>
+        <v>0.348</v>
       </c>
       <c r="G7" t="n">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="H7" t="n">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>opp QB: fill-in QB (Tanner McKee)</t>
+          <t>fill-in QB (Tanner McKee) red-team downgrade</t>
         </is>
       </c>
     </row>
@@ -8682,16 +8732,16 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.321</v>
+        <v>0.294</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.304</v>
+        <v>0.279</v>
       </c>
       <c r="G8" t="n">
-        <v>212</v>
+        <v>240</v>
       </c>
       <c r="H8" t="n">
-        <v>249</v>
+        <v>281</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>0.95</v>
@@ -8724,16 +8774,16 @@
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.272</v>
+        <v>0.266</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.258</v>
+        <v>0.252</v>
       </c>
       <c r="G9" t="n">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="H9" t="n">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>0.95</v>
@@ -8747,7 +8797,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Darius Cooper</t>
+          <t>Saquon Barkley</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8762,34 +8812,34 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.251</v>
+        <v>0.233</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.251</v>
+        <v>0.233</v>
       </c>
       <c r="G10" t="n">
-        <v>299</v>
+        <v>329</v>
       </c>
       <c r="H10" t="n">
-        <v>347</v>
+        <v>381</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>fill-in QB (Tanner McKee) red-team downgrade</t>
+          <t>fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Zach Ertz</t>
+          <t>Darius Cooper</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8804,20 +8854,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.224</v>
+        <v>0.229</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.224</v>
+        <v>0.229</v>
       </c>
       <c r="G11" t="n">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="H11" t="n">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>1</v>
@@ -8850,16 +8900,16 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>0.219</v>
+        <v>0.215</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>0.219</v>
+        <v>0.215</v>
       </c>
       <c r="G12" t="n">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="H12" t="n">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>1</v>
@@ -8873,7 +8923,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Makai Lemon</t>
+          <t>Zach Ertz</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8888,76 +8938,76 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.216</v>
+        <v>0.198</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0.216</v>
+        <v>0.198</v>
       </c>
       <c r="G13" t="n">
-        <v>364</v>
+        <v>405</v>
       </c>
       <c r="H13" t="n">
-        <v>420</v>
+        <v>465</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>fill-in QB (Tanner McKee)</t>
+          <t>fill-in QB (Tanner McKee) red-team downgrade</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jake Ferguson</t>
+          <t>Makai Lemon</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>0.18</v>
+        <v>0.195</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>0.18</v>
+        <v>0.195</v>
       </c>
       <c r="G14" t="n">
-        <v>455</v>
+        <v>413</v>
       </c>
       <c r="H14" t="n">
-        <v>522</v>
+        <v>474</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>opp QB: fill-in QB (Tanner McKee)</t>
+          <t>fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dak Prescott</t>
+          <t>Jake Ferguson</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8972,20 +9022,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.146</v>
+        <v>0.183</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0.146</v>
+        <v>0.183</v>
       </c>
       <c r="G15" t="n">
-        <v>583</v>
+        <v>445</v>
       </c>
       <c r="H15" t="n">
-        <v>665</v>
+        <v>511</v>
       </c>
       <c r="I15" s="6" t="n">
         <v>1</v>
@@ -8999,7 +9049,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Tyler Goodson</t>
+          <t>Dak Prescott</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9014,20 +9064,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>0.128</v>
+        <v>0.149</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>0.128</v>
+        <v>0.149</v>
       </c>
       <c r="G16" t="n">
-        <v>679</v>
+        <v>571</v>
       </c>
       <c r="H16" t="n">
-        <v>773</v>
+        <v>652</v>
       </c>
       <c r="I16" s="6" t="n">
         <v>1</v>
@@ -9041,7 +9091,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hunter Luepke</t>
+          <t>Tyler Goodson</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9060,16 +9110,16 @@
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>0.062</v>
+        <v>0.131</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.062</v>
+        <v>0.131</v>
       </c>
       <c r="G17" t="n">
-        <v>1509</v>
+        <v>664</v>
       </c>
       <c r="H17" t="n">
-        <v>1702</v>
+        <v>756</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>1</v>
@@ -9083,49 +9133,49 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Jonathan Mingo</t>
+          <t>Marquise Brown</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>WR</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>0.06</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>0.06</v>
+        <v>0.08900000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>1567</v>
+        <v>970</v>
       </c>
       <c r="H18" t="n">
-        <v>1767</v>
+        <v>1099</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>opp QB: fill-in QB (Tanner McKee)</t>
+          <t>fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Luke Schoonmaker</t>
+          <t>Hunter Luepke</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9140,20 +9190,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.06</v>
+        <v>0.063</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>0.06</v>
+        <v>0.063</v>
       </c>
       <c r="G19" t="n">
-        <v>1567</v>
+        <v>1480</v>
       </c>
       <c r="H19" t="n">
-        <v>1767</v>
+        <v>1669</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>1</v>
@@ -9167,7 +9217,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Brevyn Spann-Ford</t>
+          <t>Jonathan Mingo</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9182,7 +9232,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
@@ -9209,22 +9259,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Elijah Moore</t>
+          <t>Luke Schoonmaker</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
@@ -9244,24 +9294,24 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>fill-in QB (Tanner McKee)</t>
+          <t>opp QB: fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Johnny Mundt</t>
+          <t>Brevyn Spann-Ford</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>PHI</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>DAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -9286,14 +9336,14 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>fill-in QB (Tanner McKee)</t>
+          <t>opp QB: fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Britain Covey</t>
+          <t>Elijah Moore</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9312,19 +9362,19 @@
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.021</v>
+        <v>0.06</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="G23" t="n">
-        <v>4733</v>
+        <v>1567</v>
       </c>
       <c r="H23" t="n">
-        <v>5313</v>
+        <v>1767</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -9332,85 +9382,104 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Johnny Mundt</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1567</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1767</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>fill-in QB (Tanner McKee)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>2+ TD (top 10)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>player</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>team</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>opp</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>prob</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>fair</t>
         </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Javonte Williams</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="n">
-        <v>0.254</v>
-      </c>
-      <c r="E27" t="n">
-        <v>293</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dameon Pierce</t>
+          <t>Javonte Williams</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
       <c r="D28" s="6" t="n">
-        <v>0.092</v>
+        <v>0.254</v>
       </c>
       <c r="E28" t="n">
-        <v>985</v>
+        <v>293</v>
       </c>
     </row>
     <row r="29">
@@ -9430,16 +9499,16 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>0.064</v>
+        <v>0.068</v>
       </c>
       <c r="E29" t="n">
-        <v>1467</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dallas Goedert</t>
+          <t>Dameon Pierce</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9453,62 +9522,62 @@
         </is>
       </c>
       <c r="D30" s="6" t="n">
-        <v>0.052</v>
+        <v>0.062</v>
       </c>
       <c r="E30" t="n">
-        <v>1812</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>George Pickens</t>
+          <t>Dallas Goedert</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
       <c r="D31" s="6" t="n">
-        <v>0.038</v>
+        <v>0.044</v>
       </c>
       <c r="E31" t="n">
-        <v>2561</v>
+        <v>2151</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Darius Cooper</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
       <c r="D32" s="6" t="n">
-        <v>0.032</v>
+        <v>0.03700000000000001</v>
       </c>
       <c r="E32" t="n">
-        <v>3070</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Zach Ertz</t>
+          <t>Darius Cooper</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9525,157 +9594,157 @@
         <v>0.026</v>
       </c>
       <c r="E33" t="n">
-        <v>3776</v>
+        <v>3761</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ryan Flournoy</t>
+          <t>Saquon Barkley</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
           <t>DAL</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>PHI</t>
         </is>
       </c>
       <c r="D34" s="6" t="n">
         <v>0.025</v>
       </c>
       <c r="E34" t="n">
-        <v>3916</v>
+        <v>3845</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Makai Lemon</t>
+          <t>Ryan Flournoy</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
       <c r="D35" s="6" t="n">
-        <v>0.022</v>
+        <v>0.021</v>
       </c>
       <c r="E35" t="n">
-        <v>4530</v>
+        <v>4551</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jake Ferguson</t>
+          <t>Zach Ertz</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="D36" s="6" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4562</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Makai Lemon</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="D36" s="6" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="E36" t="n">
-        <v>5835</v>
-      </c>
-    </row>
-    <row r="37"/>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="E37" t="n">
+        <v>4731</v>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>First TD (top 10)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>player</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>team</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>opp</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>prob</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>fair</t>
         </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Javonte Williams</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="n">
-        <v>0.195</v>
-      </c>
-      <c r="E40" t="n">
-        <v>412</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Dameon Pierce</t>
+          <t>Javonte Williams</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
       <c r="D41" s="6" t="n">
-        <v>0.104</v>
+        <v>0.196</v>
       </c>
       <c r="E41" t="n">
-        <v>865</v>
+        <v>410</v>
       </c>
     </row>
     <row r="42">
@@ -9695,16 +9764,16 @@
         </is>
       </c>
       <c r="D42" s="6" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="E42" t="n">
-        <v>1075</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dallas Goedert</t>
+          <t>Dameon Pierce</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -9718,62 +9787,62 @@
         </is>
       </c>
       <c r="D43" s="6" t="n">
-        <v>0.075</v>
+        <v>0.083</v>
       </c>
       <c r="E43" t="n">
-        <v>1236</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>George Pickens</t>
+          <t>Dallas Goedert</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
       <c r="D44" s="6" t="n">
-        <v>0.062</v>
+        <v>0.068</v>
       </c>
       <c r="E44" t="n">
-        <v>1515</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Darius Cooper</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>DAL</t>
-        </is>
-      </c>
       <c r="D45" s="6" t="n">
-        <v>0.057</v>
+        <v>0.061</v>
       </c>
       <c r="E45" t="n">
-        <v>1669</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Zach Ertz</t>
+          <t>Saquon Barkley</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -9787,86 +9856,109 @@
         </is>
       </c>
       <c r="D46" s="6" t="n">
-        <v>0.05</v>
+        <v>0.051</v>
       </c>
       <c r="E46" t="n">
-        <v>1920</v>
+        <v>1843</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ryan Flournoy</t>
+          <t>Darius Cooper</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>PHI</t>
-        </is>
-      </c>
       <c r="D47" s="6" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="E47" t="n">
-        <v>1957</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Makai Lemon</t>
+          <t>Ryan Flournoy</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
           <t>PHI</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>DAL</t>
         </is>
       </c>
       <c r="D48" s="6" t="n">
         <v>0.047</v>
       </c>
       <c r="E48" t="n">
-        <v>2031</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Jake Ferguson</t>
+          <t>Zach Ertz</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
           <t>DAL</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="D49" s="6" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2191</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Makai Lemon</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>PHI</t>
         </is>
       </c>
-      <c r="D49" s="6" t="n">
-        <v>0.039</v>
-      </c>
-      <c r="E49" t="n">
-        <v>2439</v>
-      </c>
-    </row>
-    <row r="50"/>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Sneaky longshots (8% to 25% anytime, active 90%+): Zach Ertz (PHI) 22% fair +346, take at +400+; Ryan Flournoy (DAL) 22% fair +357, take at +412+; Makai Lemon (PHI) 22% fair +364, take at +420+; Jake Ferguson (DAL) 18% fair +455, take at +522+; Dak Prescott (DAL) 15% fair +583, take at +665+; Tyler Goodson (DAL) 13% fair +679, take at +773+</t>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="E50" t="n">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Sneaky longshots (8% to 25% anytime, active 90%+): Saquon Barkley (PHI) 23% fair +329, take at +381+; Darius Cooper (PHI) 23% fair +338, take at +390+; Ryan Flournoy (DAL) 22% fair +364, take at +420+; Zach Ertz (PHI) 20% fair +405, take at +465+; Makai Lemon (PHI) 20% fair +413, take at +474+; Jake Ferguson (DAL) 18% fair +445, take at +511+; Dak Prescott (DAL) 15% fair +571, take at +652+; Tyler Goodson (DAL) 13% fair +664, take at +756+; Marquise Brown (PHI) 9% fair +970, take at +1099+</t>
         </is>
       </c>
     </row>
@@ -10011,13 +10103,13 @@
         <v>5.5</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>1</v>
+        <v>0.96</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="I5" t="n">
-        <v>-298</v>
+        <v>-267</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -10053,7 +10145,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dameon Pierce</t>
+          <t>Saquon Barkley</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -10063,24 +10155,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>18.5</v>
+        <v>65.5</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.98</v>
+        <v>0.91</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="I6" t="n">
-        <v>-284</v>
+        <v>-238</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -10112,7 +10204,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tanner McKee</t>
+          <t>Dameon Pierce</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -10126,20 +10218,20 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.5</v>
+        <v>18.5</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.77</v>
+        <v>0.88</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.64</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>-175</v>
+        <v>-221</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -10191,10 +10283,10 @@
         <v>0.73</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="I8" t="n">
-        <v>-160</v>
+        <v>-159</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -10250,7 +10342,7 @@
         <v>0.65</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="I9" t="n">
         <v>-135</v>
@@ -10312,7 +10404,7 @@
         <v>0.57</v>
       </c>
       <c r="I10" t="n">
-        <v>-134</v>
+        <v>-135</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -10353,7 +10445,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>pass_yds</t>
+          <t>pass_cmp</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -10362,16 +10454,16 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>202.5</v>
+        <v>20.5</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.61</v>
+        <v>0.59</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="I11" t="n">
-        <v>-125</v>
+        <v>-119</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -10380,7 +10472,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -10412,7 +10504,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>rush_att</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -10421,7 +10513,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>16.5</v>
+        <v>64.5</v>
       </c>
       <c r="G12" s="6" t="n">
         <v>0.58</v>
@@ -10430,11 +10522,11 @@
         <v>0.54</v>
       </c>
       <c r="I12" t="n">
-        <v>-117</v>
+        <v>-118</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -10466,21 +10558,21 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tanner McKee</t>
+          <t>Javonte Williams</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>pass_cmp</t>
+          <t>rush_att</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>20.5</v>
+        <v>16.5</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>0.58</v>
@@ -10493,12 +10585,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -10508,7 +10600,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>fill-in QB (Tanner McKee)</t>
+          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
@@ -10525,39 +10617,39 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Javonte Williams</t>
+          <t>Tanner McKee</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>pass_yds</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>64.5</v>
+        <v>203.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>0.58</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I14" t="n">
-        <v>-117</v>
+        <v>-113</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -10567,7 +10659,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
+          <t>fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
@@ -10643,12 +10735,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dak Prescott</t>
+          <t>Tanner McKee</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>pass_cmp</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -10657,25 +10749,25 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>24.5</v>
+        <v>3.5</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="H16" s="6" t="n">
         <v>0.51</v>
       </c>
       <c r="I16" t="n">
-        <v>-104</v>
+        <v>-105</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -10685,7 +10777,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
+          <t>fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
@@ -10702,43 +10794,39 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Saquon Barkley</t>
+          <t>Dak Prescott</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>pass_cmp</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
+        <v>24.5</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>0.51</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>-103</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -10748,7 +10836,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>fill-in QB (Tanner McKee)</t>
+          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>

</xml_diff>